<commit_message>
Sync WP Olympiad 1.0.3 and establish ongoing release publishing
</commit_message>
<xml_diff>
--- a/templates/questions_template.xlsx
+++ b/templates/questions_template.xlsx
@@ -259,7 +259,7 @@
             <family val="2"/>
           </rPr>
           <t>[extra]
-Пары key=value через «;». Ключи: min, max, step, extra_letters, audio_url, scoring, mistakes, mode, distractors, min_words, max_words, keywords, min_keywords, match, typo, shuffle, case_sensitive.</t>
+Пары key=value через «;». Ключи: min, max, step, extra_letters, audio_url, scoring, mistakes, mode, distractors, min_words, max_words, keywords, min_keywords, match, typo, shuffle, case_sensitive, show_points (1 — показывать баллы за это задание, по умолчанию они скрыты).</t>
         </r>
       </text>
     </comment>
@@ -552,13 +552,13 @@
     <t>4.</t>
   </si>
   <si>
-    <t>Для проверки нажмите «✔ Проверить данные» (в файле .xlsm) — макрос подсветит ошибки.</t>
+    <t>Для проверки используйте «Проверить файл заданий» в WordPress — проверка не меняет базу.</t>
   </si>
   <si>
     <t>5.</t>
   </si>
   <si>
-    <t>Сохраните файл как questions.csv в кодировке UTF-8 или нажмите «📥 Экспорт в CSV».</t>
+    <t>Сохраните заполненную книгу как Мои_вопросы.xlsx. Макросы и преобразование в CSV не требуются.</t>
   </si>
   <si>
     <t>6.</t>
@@ -711,7 +711,7 @@
     <t>extra</t>
   </si>
   <si>
-    <t>Пары key=value через «;». Ключи: min, max, step, extra_letters, audio_url, scoring, mistakes, mode, distractors, min_words, max_words, keywords, min_keywords, match, typo, shuffle, case_sensitive.</t>
+    <t>Пары key=value через «;». Ключи: min, max, step, extra_letters, audio_url, scoring, mistakes, mode, distractors, min_words, max_words, keywords, min_keywords, match, typo, shuffle, case_sensitive, show_points (1 — показывать баллы за это задание, по умолчанию они скрыты).</t>
   </si>
   <si>
     <t>3. ВСЕ ТИПЫ ЗАДАНИЙ</t>

</xml_diff>